<commit_message>
fix(ledger): A-4 debe su convenio — el aporte al tanque se lo habia pagado
Los dos yapes de A-4 del 07/07 no son el mismo pago repetido: S/136 es deuda y
S/100 dice "tanque" en el propio mensaje. motor_matching dejo CONCEPTO vacio,
los 236 entraron juntos y la cascada se comio el aporte como pago de deuda.

Con los 136 reales la cascada llega hasta ACUERDOS y CONVENIO queda impago:
136 = 31 agua + 30 MULTA + 75 ACUERDOS. planilla_cobrado ya decia SALDO 75
(5_cobranza lee aportes_tanque_manuales antes de la cascada); el ledger no se
habia enterado.

Se borran las 5 filas de A-4 CONVENIO posteriores a la siembra: 2 PAGO fantasma
y los 3 AJUSTE con que el sistema se corregia a si mismo. Queda el CARGO, saldo
75. Mismo criterio que la limpieza del 06/08.

1491 -> 1486 eventos · 0 saldos negativos · vista regenerada · tests OK.

La secretaria ya habia reclamado que A-4 debia. Tenia razon.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shared/vista_seguimiento_pueblo.xlsx
+++ b/shared/vista_seguimiento_pueblo.xlsx
@@ -24556,14 +24556,20 @@
       <c r="F4" s="8" t="n">
         <v>75</v>
       </c>
-      <c r="G4" s="10" t="n">
-        <v>75</v>
-      </c>
-      <c r="H4" s="7" t="n">
-        <v>150</v>
-      </c>
-      <c r="I4" s="11" t="n">
-        <v>0</v>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -30741,10 +30747,10 @@
         <v>0</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="M4" s="11" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5">

</xml_diff>